<commit_message>
Final version with login, voice output, and recommendations
</commit_message>
<xml_diff>
--- a/prediction_history.xlsx
+++ b/prediction_history.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,6 +464,16 @@
           <t>GDD</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>User Name</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>User Email</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -497,6 +507,8 @@
       <c r="G2" t="n">
         <v>18</v>
       </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -530,6 +542,8 @@
       <c r="G3" t="n">
         <v>18</v>
       </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -563,6 +577,8 @@
       <c r="G4" t="n">
         <v>18</v>
       </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -595,6 +611,481 @@
       </c>
       <c r="G5" t="n">
         <v>18</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>20-07-2026 14:29:50</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>healthy8.jpg</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>HEALTHY</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>100</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Larva Stage</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>19</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Rajendran R</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>rr8511142@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>20-07-2026 14:35:10</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>healthy50.jpg</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>HEALTHY</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Larva Stage</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>18</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Rajendran R</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>rr8511142@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>20-07-2026 14:45:27</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>healthy14.jpg</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>HEALTHY</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>99.84999999999999</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Larva Stage</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>20</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Rajendran R</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>rr8511142@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>20-07-2026 15:03:20</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>healthy8.jpg</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>HEALTHY</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Larva Stage</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Rajendran R</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>rr8511142@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>20-07-2026 15:03:43</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>infected_mango.jpg</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>INFECTED</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>100</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Larva Stage</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>21</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Rajendran R</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>rr8511142@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>20-07-2026 15:04:36</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>infected63.jpg</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>INFECTED</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>99.87</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Larva Stage</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>18</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Rajendran R</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>rr8511142@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>20-07-2026 15:09:02</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>infected13.jpg</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>INFECTED</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>99.98999999999999</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Pupa Stage</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Rajendran R</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>rr8511142@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>20-07-2026 15:23:04</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>infected6.jpg</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>INFECTED</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>98.95</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Pupa Stage</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Rajendran R</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>rr8511142@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>20-07-2026 15:35:43</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>infected108.jpg</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>INFECTED</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>100</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Larva Stage</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>24</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Rajendran R</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>rr8511142@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>20-07-2026 15:42:26</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>healthy3.jpg</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>HEALTHY</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>99.95999999999999</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Egg Stage</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Rajendran R</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>rr8511142@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>20-07-2026 20:44:45</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>healthy8.jpg</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>HEALTHY</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>100</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Larva Stage</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Rajendran R</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>rr8511142@gmail.com</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>